<commit_message>
Daily job scrape update
</commit_message>
<xml_diff>
--- a/data/job_tracker.xlsx
+++ b/data/job_tracker.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I17"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -630,12 +630,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>BearingPoint</t>
+          <t>Agile Robots</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -645,7 +645,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>(Senior) Consultant / Architect ServiceNow Banking &amp; Insurance (m/w/d) Berlin, Düsseldorf, Frankfurt am Main, Hamburg, Leipzig, München, Stuttgart, Walldorf</t>
+          <t>Senior Project Manager (all genders)</t>
         </is>
       </c>
       <c r="E5" t="n">
@@ -653,29 +653,29 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Berlin, DE; Düsseldorf, DE; Frankfurt am Main, DE; Hamburg, DE; Leipzig, DE; München, DE; Stuttgart, DE; Walldorf, DE</t>
+          <t>Munich, Bavaria, Germany</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>https://www.bearingpoint.com/de-de/karriere/stellenangebote/angebot/?id=T7549597</t>
+          <t>https://job-boards.eu.greenhouse.io/agilerobotsse/jobs/4990647101</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Related role</t>
+          <t>Direct role</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Responsibilities: delivery, transformation</t>
+          <t>Title: project manager</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -690,11 +690,11 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Senior Project Manager (all genders)</t>
+          <t>(Senior) Technical Program Manager (m/f/d)</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -703,7 +703,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>https://job-boards.eu.greenhouse.io/agilerobotsse/jobs/4990647101</t>
+          <t>https://job-boards.eu.greenhouse.io/agilerobotsse/jobs/4996481101</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -713,19 +713,19 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Title: project manager</t>
+          <t>Title: program manager</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Celonis</t>
+          <t>Proxima Fusion</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -735,480 +735,120 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Senior Business Transformation &amp; Process Optimisation Consultant - Aviation/Logistics</t>
+          <t>Site Development Program Manager</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Munich, Germany</t>
+          <t>Munich</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/celonis/jobs/8015653003?gh_jid=8015653003</t>
+          <t>https://jobs.ashbyhq.com/proxima-fusion/db5bc40c-aa3e-4735-94e7-096a556dd55d</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Related role</t>
+          <t>Direct role</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Responsibilities: delivery, stakeholders, transformation</t>
+          <t>Title: program manager</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>2026-10-08</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Celonis</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Munich</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Senior Digital Transformation &amp; Process Optimisation Consultant - CPG/Retail</t>
-        </is>
-      </c>
-      <c r="E8" t="n">
-        <v>4</v>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>Munich, Germany</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>https://job-boards.greenhouse.io/celonis/jobs/8016417003?gh_jid=8016417003</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>Related role</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>Responsibilities: delivery, stakeholders, transformation</t>
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Isar Aerospace</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>LCA &amp; Environmental Data Specialist (f/m/d)</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Parsdorf, Bavaria, Germany</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>https://job-boards.eu.greenhouse.io/isaraerospace/jobs/5009959101</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Direct role</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>Title: environmental</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>2026-10-07</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Celonis</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Munich</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Senior Management &amp; Technology Consultant - Aviation/Logistics</t>
-        </is>
-      </c>
-      <c r="E9" t="n">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Isar Aerospace</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Environmental Management Specialist (f/m/d)</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>Munich, Germany</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>https://job-boards.greenhouse.io/celonis/jobs/8015654003?gh_jid=8015654003</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>Related role</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>Responsibilities: delivery, stakeholders, transformation</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>2026-10-08</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Celonis</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Munich</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Senior Management &amp; Technology Consultant - CPG/Retail - CPG/Retail</t>
-        </is>
-      </c>
-      <c r="E10" t="n">
-        <v>4</v>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>Munich, Germany</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>https://job-boards.greenhouse.io/celonis/jobs/8016657003?gh_jid=8016657003</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>Related role</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>Responsibilities: delivery, stakeholders, transformation</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>2026-10-12</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Celonis</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Munich</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>Senior Management &amp; Technology Consultant - Growth &amp; Scale Accounts</t>
-        </is>
-      </c>
-      <c r="E11" t="n">
-        <v>4</v>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>Munich, Germany</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>https://job-boards.greenhouse.io/celonis/jobs/8026730003?gh_jid=8026730003</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>Related role</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>Responsibilities: governance, stakeholders, transformation</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>2026-10-07</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Celonis</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Munich</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>Senior Process Intelligence &amp; Supply Chain Transformation Consultant - Aviation/Logistics</t>
-        </is>
-      </c>
-      <c r="E12" t="n">
-        <v>4</v>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>Munich, Germany</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>https://job-boards.greenhouse.io/celonis/jobs/8015655003?gh_jid=8015655003</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>Related role</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>Responsibilities: delivery, stakeholders, transformation</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>2026-10-08</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Celonis</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Munich</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>Senior Process Intelligence &amp; Supply Chain Transformation Consultant - CPG/Retail</t>
-        </is>
-      </c>
-      <c r="E13" t="n">
-        <v>4</v>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>Munich, Germany</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>https://job-boards.greenhouse.io/celonis/jobs/8016658003?gh_jid=8016658003</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>Related role</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>Responsibilities: delivery, stakeholders, transformation</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>2026-10-12</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Celonis</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Munich</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>Senior Process Optimisation Consultant - Growth &amp; Scale Accounts</t>
-        </is>
-      </c>
-      <c r="E14" t="n">
-        <v>4</v>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>Munich, Germany</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>https://job-boards.greenhouse.io/celonis/jobs/8026747003?gh_jid=8026747003</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>Related role</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>Responsibilities: governance, stakeholders, transformation</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>2026-10-02</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Agile Robots</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Munich</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>(Senior) Technical Program Manager (m/f/d)</t>
-        </is>
-      </c>
-      <c r="E15" t="n">
-        <v>4</v>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>Munich, Bavaria, Germany</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>https://job-boards.eu.greenhouse.io/agilerobotsse/jobs/4996481101</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Parsdorf, Bavaria, Germany</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>https://job-boards.eu.greenhouse.io/isaraerospace/jobs/5009977101</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
         <is>
           <t>Direct role</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>Title: program manager</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>2026-10-13</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Proxima Fusion</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Munich</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>Site Development Program Manager</t>
-        </is>
-      </c>
-      <c r="E16" t="n">
-        <v>3</v>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>Munich</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>https://jobs.ashbyhq.com/proxima-fusion/db5bc40c-aa3e-4735-94e7-096a556dd55d</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>Direct role</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>Title: program manager</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>2026-09-30</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Isar Aerospace</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>Munich</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>MES Delivery Manager / Project Manager (m/f/d)</t>
-        </is>
-      </c>
-      <c r="E17" t="n">
-        <v>8</v>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>Parsdorf, Bavaria, Germany</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>https://job-boards.eu.greenhouse.io/isaraerospace/jobs/4989582101</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>Direct role</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>Title: project manager</t>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>Title: environmental</t>
         </is>
       </c>
     </row>

</xml_diff>